<commit_message>
[34차] Stage1Group 완성 + 전체 씬 안정화 + Make it Right 구조 개선
이번 커밋은 Stage1Group을 완성하고, 기존 씬들의 안정화 작업을 진행한 커밋입니다.

**주요 변경 내용:**

- Stage1Group 완성
  - Stage1-1 (NPC 대화 영역)과 Stage1-2 (호박 획득 영역) 구현
  - Moran 이동 시스템 (Idle / Walking / Running) 완성
  - StageName 데이터 드리븐 표시 + 자연스러운 등장/사라짐 연출
  - NPC 상호작용, 퀘스트 진행, 호박 획득 흐름 연결

- 전체 씬 안정화
  - 1st_Road_to_Stage1 HUD, 튜토리얼, CookingGroup 안정화
  - Senario1Group Moran 오브젝트 복구 및 위치 조정
  - 여러 씬에서 발생하던 참조/활성화/튜토리얼 진행 버그 수정

- Make it Right 구조 개선
  - Stage1Group을 이후 Stage2, Stage3, Stage4, FinalStage까지 거의 동일하게 재사용할 수 있는 포맷으로 정리
  - Controller 역할 분리 강화 (장면 지휘 중심)
  - 컴포넌트 기반 구조로 리팩토링 진행

**이번 작업으로:**
- Stage1Group이 플레이 가능한 수준으로 완성됨
- 기존 씬들의 안정성 대폭 향상
- 이후 스테이지 제작 시 재사용하기 좋은 기반 구조 마련
- Make it Work에서 Make it Right 방향으로 한 단계 진전

**다음 목표:**
- Stage2Group ~ Stage4Group 제작
- FinalStageGroup 구현
- 요리 시스템 세밀 조정 및 데이터 드리븐 강화
- 인벤토리/퀘스트 UI 완성도 향상

오늘 Stage1Group 완성과 전체 안정화 작업을 마무리했습니다.
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/OO_Dialogue.xlsx
+++ b/JsonConverter/ExcelFiles/OO_Dialogue.xlsx
@@ -1002,583 +1002,583 @@
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
+    <r>
+      <t>“</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="돋움"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>허어</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="돋움"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>눈물이</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="돋움"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>앞을</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="돋움"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>가리는구려</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">…… </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="돋움"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>이</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="돋움"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>은혜를</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="돋움"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>어찌</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="돋움"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="돋움"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>갚아야</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="돋움"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>할지</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="돋움"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>모르겠소</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="돋움"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>비록</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="돋움"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>지금은</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="돋움"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>척박해진</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="돋움"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>땅이나</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="돋움"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>매서운</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="돋움"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>추위도</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="돋움"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>잊게</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="돋움"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>만드는</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="돋움"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>우리</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="돋움"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>마을의</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="돋움"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>오랜</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="돋움"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>특산물인</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="돋움"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>청양고추라오</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="돋움"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>모란님의</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="돋움"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>앞날에</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="돋움"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>작게나마</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="돋움"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>보탬이</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="돋움"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>되길</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="돋움"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>바라오</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>.”</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
     <t>character_VillageChief_02</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>“</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>허어</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>눈물이</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>앞을</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>가리는구려</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">…… </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>이</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>은혜를</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>어찌</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>다</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>갚아야</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>할지</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>모르겠소</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>비록</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>지금은</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>척박해진</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>땅이나</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>매서운</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>추위도</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>잊게</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>만드는</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>우리</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>마을의</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>오랜</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>특산물인</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>청양고추라오</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>모란님의</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>앞날에</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>작게나마</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>보탬이</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>되길</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>바라오</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>.”</t>
-    </r>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
 </sst>
@@ -2420,13 +2420,13 @@
     </row>
     <row r="20" spans="1:5" ht="15.75" customHeight="1">
       <c r="A20" s="8" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B20" s="15" t="s">
         <v>53</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="15.75" customHeight="1">
@@ -3476,6 +3476,6 @@
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
[42차] Stage3 BGM 넣기 + Stage4 가는 길과 진입 1차 정리
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/OO_Dialogue.xlsx
+++ b/JsonConverter/ExcelFiles/OO_Dialogue.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="108">
   <si>
     <t>대사 ID</t>
   </si>
@@ -293,9 +293,6 @@
     <t>"나는 이곳에 남아 흩어진 민심을 바로잡고 왕실의 어둠을 살필 테니, 춘양 자네는 저들과 함께 고통받는 세상을 구하는 아름다운 여정을 계속 이어가 주시게. 내 너희의 여정에 보탬이 되길 바라며 이 쌀과 꿀단지를 내어주니, 부디 요긴하게 쓰이길 바란다."</t>
   </si>
   <si>
-    <t>character_Chunyang_09</t>
-  </si>
-  <si>
     <t>"(흐르는 눈물을 닦고 입을 가리며 수줍게 미소 짓는다) 나으리의 깊은 뜻을 어찌 거스르겠나이다. 서방님께서 주신 영약과 이 비단결 같은 동료들이 있으니, 제 앞길에 두려울 것이 없사옵니다. 부디 몸조심하시옵소서. 이 모험의 끝에서, 더 밝아진 세상에서 반드시 다시 만나기를 기약하겠나이다."</t>
   </si>
   <si>
@@ -334,6 +331,33 @@
   <si>
     <t>character_Sangun_04</t>
     <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>character_Chunyang_09</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>character_</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Turtle_01</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>거북이</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>“아이고, 이보시오 요리사 양반! 용왕님의 병을 고치려면 저 얄미운 토끼 녀석의 간이 절실히 필요하다오. 달리기 경주로 담판을 지으려 했건만, 발이 어찌나 빠른지 등껍질이 터지도록 뛰어도 도저히 잡을 수가 없으니 내 신세가 처량하구려…….”</t>
   </si>
 </sst>
 </file>
@@ -1392,24 +1416,24 @@
     </row>
     <row r="36" spans="1:8" ht="15.75" customHeight="1">
       <c r="A36" s="26" t="s">
-        <v>92</v>
+        <v>104</v>
       </c>
       <c r="B36" s="25" t="s">
         <v>27</v>
       </c>
       <c r="C36" s="26" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="37" spans="1:8" ht="15.75" customHeight="1">
       <c r="A37" s="28" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B37" s="28" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C37" s="28" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D37" s="29"/>
       <c r="E37" s="29"/>
@@ -1419,16 +1443,16 @@
     </row>
     <row r="38" spans="1:8" ht="15.75" customHeight="1">
       <c r="A38" s="28" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B38" s="28" t="s">
+        <v>93</v>
+      </c>
+      <c r="C38" s="28" t="s">
         <v>94</v>
       </c>
-      <c r="C38" s="28" t="s">
+      <c r="D38" s="29" t="s">
         <v>95</v>
-      </c>
-      <c r="D38" s="29" t="s">
-        <v>96</v>
       </c>
       <c r="E38" s="29"/>
       <c r="F38" s="29"/>
@@ -1437,16 +1461,16 @@
     </row>
     <row r="39" spans="1:8" ht="15.75" customHeight="1">
       <c r="A39" s="28" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B39" s="28" t="s">
         <v>18</v>
       </c>
       <c r="C39" s="28" t="s">
+        <v>96</v>
+      </c>
+      <c r="D39" s="29" t="s">
         <v>97</v>
-      </c>
-      <c r="D39" s="29" t="s">
-        <v>98</v>
       </c>
       <c r="E39" s="29"/>
       <c r="F39" s="29"/>
@@ -1455,13 +1479,13 @@
     </row>
     <row r="40" spans="1:8" ht="15.75" customHeight="1">
       <c r="A40" s="28" t="s">
+        <v>97</v>
+      </c>
+      <c r="B40" s="28" t="s">
+        <v>93</v>
+      </c>
+      <c r="C40" s="28" t="s">
         <v>98</v>
-      </c>
-      <c r="B40" s="28" t="s">
-        <v>94</v>
-      </c>
-      <c r="C40" s="28" t="s">
-        <v>99</v>
       </c>
       <c r="D40" s="29"/>
       <c r="E40" s="29"/>
@@ -1471,13 +1495,13 @@
     </row>
     <row r="41" spans="1:8" ht="15.75" customHeight="1">
       <c r="A41" s="28" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B41" s="28" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C41" s="28" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D41" s="29"/>
       <c r="E41" s="29"/>
@@ -1495,7 +1519,17 @@
       <c r="G42" s="27"/>
       <c r="H42" s="27"/>
     </row>
-    <row r="43" spans="1:8" ht="15.75" customHeight="1"/>
+    <row r="43" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A43" s="26" t="s">
+        <v>105</v>
+      </c>
+      <c r="B43" s="25" t="s">
+        <v>106</v>
+      </c>
+      <c r="C43" s="13" t="s">
+        <v>107</v>
+      </c>
+    </row>
     <row r="44" spans="1:8" ht="15.75" customHeight="1"/>
     <row r="45" spans="1:8" ht="15.75" customHeight="1"/>
     <row r="46" spans="1:8" ht="15.75" customHeight="1"/>

</xml_diff>